<commit_message>
UI changes for Credit & Debit card for all pages
</commit_message>
<xml_diff>
--- a/KatalonData/IVT/IVT_Login.xlsx
+++ b/KatalonData/IVT/IVT_Login.xlsx
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="37">
   <si>
     <t>Result</t>
   </si>
@@ -285,6 +285,21 @@
   </si>
   <si>
     <t>Fri Sep 18 12:55:17 IST 2026</t>
+  </si>
+  <si>
+    <t>Mon Sep 28 17:35:43 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Sep 29 12:05:08 IST 2026</t>
+  </si>
+  <si>
+    <t>Tue Sep 29 20:02:46 IST 2026</t>
+  </si>
+  <si>
+    <t>Thu Oct 01 00:31:55 IST 2026</t>
+  </si>
+  <si>
+    <t>Thu Oct 01 00:35:45 IST 2026</t>
   </si>
 </sst>
 </file>
@@ -763,7 +778,7 @@
         <v>9</v>
       </c>
       <c r="B2" s="8" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="C2" s="5" t="s">
         <v>13</v>

</xml_diff>